<commit_message>
MU FY2026Q4 report ed1 revision 1 (Jiwon review items, R20-R24)
- Narrative r4: company overview, how to read verdicts, GM beat compression,
  business-unit structure (section 5), methodology appendix
- 8 -> 16 charts, each shown once, numbered in page order; bold headings;
  reader-facing tables and captions (no internal IDs or raw codes)
- Gates 62 PASS, forecast tests 577 PASS; KO 24p / EN 26p
- No change to numbers, RLE rules or frozen pre-registration
- Not investment advice
</commit_message>
<xml_diff>
--- a/forecast/reports/mu_report_fy2026q4_ed1_data.xlsx
+++ b/forecast/reports/mu_report_fy2026q4_ed1_data.xlsx
@@ -106,7 +106,9 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -498,10 +500,10 @@
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc. (NASDAQ: MU)</t>
+          <t>MICRON TECHNOLOGY · NASDAQ: MU</t>
         </is>
       </c>
     </row>
@@ -539,12 +541,12 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Review &amp; Outlook — FY2026Q4 · 14주 · FY2026 53주 · 제1판</t>
+          <t>Review &amp; Outlook — FY2026Q4 · 14주 · FY2026 53주 · 제1판 개정 1</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Review &amp; Outlook — FY2026Q4 · 14 weeks · FY2026 53 weeks · First edition</t>
+          <t>Review &amp; Outlook — FY2026Q4 · 14 weeks · FY2026 53 weeks · Edition 1, Revision 1</t>
         </is>
       </c>
     </row>
@@ -675,12 +677,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>발행 직전 확인 시각(2026-10-04T14:42:00+09:00) 현재, 작성자 김지원은 Micron Technology, Inc. (MU) 주식을 보유하지 않습니다.</t>
+          <t>발행 직전 확인 시각(2026-10-05T19:07:00+09:00) 현재, 작성자 김지원은 Micron Technology, Inc. (MU) 주식을 보유하지 않습니다.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>As of the pre-publication confirmation time (2026-10-04T14:42:00+09:00), the author, Jiwon Kim, does not hold shares of Micron Technology, Inc. (MU).</t>
+          <t>As of the pre-publication confirmation time (2026-10-05T19:07:00+09:00), the author, Jiwon Kim, does not hold shares of Micron Technology, Inc. (MU).</t>
         </is>
       </c>
     </row>
@@ -737,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K760"/>
+  <dimension ref="A1:K879"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -17588,12 +17590,12 @@
       </c>
       <c r="E480" s="8" t="inlineStr">
         <is>
-          <t>CALCULATED</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F480" s="8" t="inlineStr">
         <is>
-          <t>SRC-EX991-FQ4FY26</t>
+          <t>SRC-BU-9f7e667a8224</t>
         </is>
       </c>
       <c r="G480" s="8" t="inlineStr">
@@ -27401,6 +27403,4231 @@
         </is>
       </c>
       <c r="G760" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ2-24</t>
+        </is>
+      </c>
+      <c r="B761" s="8" t="n">
+        <v>6.530000000000001</v>
+      </c>
+      <c r="C761" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D761" s="8" t="inlineStr">
+        <is>
+          <t>FQ2-24</t>
+        </is>
+      </c>
+      <c r="E761" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F761" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G761" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ3-24</t>
+        </is>
+      </c>
+      <c r="B762" s="8" t="n">
+        <v>1.399999999999999</v>
+      </c>
+      <c r="C762" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D762" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-24</t>
+        </is>
+      </c>
+      <c r="E762" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F762" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G762" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ3-24</t>
+        </is>
+      </c>
+      <c r="B763" s="8" t="n">
+        <v>8.369999999999997</v>
+      </c>
+      <c r="C763" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D763" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-24</t>
+        </is>
+      </c>
+      <c r="E763" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F763" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G763" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ4-24</t>
+        </is>
+      </c>
+      <c r="B764" s="8" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="C764" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D764" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-24</t>
+        </is>
+      </c>
+      <c r="E764" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F764" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G764" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ4-24</t>
+        </is>
+      </c>
+      <c r="B765" s="8" t="n">
+        <v>8.420000000000002</v>
+      </c>
+      <c r="C765" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D765" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-24</t>
+        </is>
+      </c>
+      <c r="E765" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F765" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G765" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ1-25</t>
+        </is>
+      </c>
+      <c r="B766" s="8" t="n">
+        <v>-0.06000000000000227</v>
+      </c>
+      <c r="C766" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D766" s="8" t="inlineStr">
+        <is>
+          <t>FQ1-25</t>
+        </is>
+      </c>
+      <c r="E766" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F766" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G766" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ1-25</t>
+        </is>
+      </c>
+      <c r="B767" s="8" t="n">
+        <v>3.119999999999997</v>
+      </c>
+      <c r="C767" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D767" s="8" t="inlineStr">
+        <is>
+          <t>FQ1-25</t>
+        </is>
+      </c>
+      <c r="E767" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F767" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G767" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ2-25</t>
+        </is>
+      </c>
+      <c r="B768" s="8" t="n">
+        <v>-0.7100000000000009</v>
+      </c>
+      <c r="C768" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D768" s="8" t="inlineStr">
+        <is>
+          <t>FQ2-25</t>
+        </is>
+      </c>
+      <c r="E768" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F768" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G768" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ2-25</t>
+        </is>
+      </c>
+      <c r="B769" s="8" t="n">
+        <v>-1.649999999999999</v>
+      </c>
+      <c r="C769" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D769" s="8" t="inlineStr">
+        <is>
+          <t>FQ2-25</t>
+        </is>
+      </c>
+      <c r="E769" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F769" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G769" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ3-25</t>
+        </is>
+      </c>
+      <c r="B770" s="8" t="n">
+        <v>2.219999999999999</v>
+      </c>
+      <c r="C770" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D770" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-25</t>
+        </is>
+      </c>
+      <c r="E770" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F770" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G770" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ3-25</t>
+        </is>
+      </c>
+      <c r="B771" s="8" t="n">
+        <v>0.9299999999999997</v>
+      </c>
+      <c r="C771" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D771" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-25</t>
+        </is>
+      </c>
+      <c r="E771" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F771" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G771" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ4-25</t>
+        </is>
+      </c>
+      <c r="B772" s="8" t="n">
+        <v>3.670000000000002</v>
+      </c>
+      <c r="C772" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D772" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-25</t>
+        </is>
+      </c>
+      <c r="E772" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F772" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G772" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ4-25</t>
+        </is>
+      </c>
+      <c r="B773" s="8" t="n">
+        <v>6.950000000000003</v>
+      </c>
+      <c r="C773" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D773" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-25</t>
+        </is>
+      </c>
+      <c r="E773" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F773" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G773" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ1-26</t>
+        </is>
+      </c>
+      <c r="B774" s="8" t="n">
+        <v>5.539999999999999</v>
+      </c>
+      <c r="C774" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D774" s="8" t="inlineStr">
+        <is>
+          <t>FQ1-26</t>
+        </is>
+      </c>
+      <c r="E774" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F774" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G774" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ1-26</t>
+        </is>
+      </c>
+      <c r="B775" s="8" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="C775" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D775" s="8" t="inlineStr">
+        <is>
+          <t>FQ1-26</t>
+        </is>
+      </c>
+      <c r="E775" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F775" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G775" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ2-26</t>
+        </is>
+      </c>
+      <c r="B776" s="8" t="n">
+        <v>7.409999999999997</v>
+      </c>
+      <c r="C776" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D776" s="8" t="inlineStr">
+        <is>
+          <t>FQ2-26</t>
+        </is>
+      </c>
+      <c r="E776" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F776" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G776" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ2-26</t>
+        </is>
+      </c>
+      <c r="B777" s="8" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="C777" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D777" s="8" t="inlineStr">
+        <is>
+          <t>FQ2-26</t>
+        </is>
+      </c>
+      <c r="E777" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F777" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G777" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ3-26</t>
+        </is>
+      </c>
+      <c r="B778" s="8" t="n">
+        <v>3.560000000000002</v>
+      </c>
+      <c r="C778" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D778" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E778" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F778" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G778" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ3-26</t>
+        </is>
+      </c>
+      <c r="B779" s="8" t="n">
+        <v>10.15000000000001</v>
+      </c>
+      <c r="C779" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D779" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E779" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F779" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G779" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_beat.FQ4-26</t>
+        </is>
+      </c>
+      <c r="B780" s="8" t="n">
+        <v>0.7561636762617781</v>
+      </c>
+      <c r="C780" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D780" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E780" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F780" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G780" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="8" t="inlineStr">
+        <is>
+          <t>derived.gm_qoq.FQ4-26</t>
+        </is>
+      </c>
+      <c r="B781" s="8" t="n">
+        <v>2.196163676261776</v>
+      </c>
+      <c r="C781" s="8" t="inlineStr">
+        <is>
+          <t>percentage_points</t>
+        </is>
+      </c>
+      <c r="D781" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E781" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F781" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G781" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="8" t="inlineStr">
+        <is>
+          <t>guidance.revenue_lo.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B782" s="8" t="n">
+        <v>49000</v>
+      </c>
+      <c r="C782" s="8" t="inlineStr">
+        <is>
+          <t>USD_million_compact</t>
+        </is>
+      </c>
+      <c r="D782" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E782" s="8" t="inlineStr">
+        <is>
+          <t>PREREG_A</t>
+        </is>
+      </c>
+      <c r="F782" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G782" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="8" t="inlineStr">
+        <is>
+          <t>guidance.revenue_hi.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B783" s="8" t="n">
+        <v>51000</v>
+      </c>
+      <c r="C783" s="8" t="inlineStr">
+        <is>
+          <t>USD_million_compact</t>
+        </is>
+      </c>
+      <c r="D783" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E783" s="8" t="inlineStr">
+        <is>
+          <t>PREREG_A</t>
+        </is>
+      </c>
+      <c r="F783" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G783" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.pricing.FQ3-26.low</t>
+        </is>
+      </c>
+      <c r="B784" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C784" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D784" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E784" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F784" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G784" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.pricing.FQ3-26.high</t>
+        </is>
+      </c>
+      <c r="B785" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="C785" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D785" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E785" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F785" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G785" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.bit_shipments.FQ3-26.low</t>
+        </is>
+      </c>
+      <c r="B786" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C786" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D786" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E786" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F786" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G786" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.bit_shipments.FQ3-26.high</t>
+        </is>
+      </c>
+      <c r="B787" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C787" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D787" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E787" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F787" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G787" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.pricing.FQ4-26.low</t>
+        </is>
+      </c>
+      <c r="B788" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C788" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D788" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E788" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F788" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G788" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.pricing.FQ4-26.high</t>
+        </is>
+      </c>
+      <c r="B789" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="C789" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D789" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E789" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F789" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G789" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.bit_shipments.FQ4-26.low</t>
+        </is>
+      </c>
+      <c r="B790" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C790" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D790" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E790" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F790" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G790" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.dram.bit_shipments.FQ4-26.high</t>
+        </is>
+      </c>
+      <c r="B791" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C791" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D791" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E791" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F791" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G791" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.pricing.FQ3-26.low</t>
+        </is>
+      </c>
+      <c r="B792" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="C792" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D792" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E792" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F792" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G792" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.pricing.FQ3-26.high</t>
+        </is>
+      </c>
+      <c r="B793" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="C793" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D793" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E793" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F793" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G793" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.bit_shipments.FQ3-26.low</t>
+        </is>
+      </c>
+      <c r="B794" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C794" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D794" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E794" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F794" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G794" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.bit_shipments.FQ3-26.high</t>
+        </is>
+      </c>
+      <c r="B795" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C795" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D795" s="8" t="inlineStr">
+        <is>
+          <t>FQ3-26</t>
+        </is>
+      </c>
+      <c r="E795" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F795" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ3-FY26</t>
+        </is>
+      </c>
+      <c r="G795" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.pricing.FQ4-26.low</t>
+        </is>
+      </c>
+      <c r="B796" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C796" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D796" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E796" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F796" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G796" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.pricing.FQ4-26.high</t>
+        </is>
+      </c>
+      <c r="B797" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="C797" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D797" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E797" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F797" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G797" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.bit_shipments.FQ4-26.low</t>
+        </is>
+      </c>
+      <c r="B798" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C798" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D798" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E798" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F798" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G798" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="8" t="inlineStr">
+        <is>
+          <t>judgment.price_bit.nand.bit_shipments.FQ4-26.high</t>
+        </is>
+      </c>
+      <c r="B799" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C799" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D799" s="8" t="inlineStr">
+        <is>
+          <t>FQ4-26</t>
+        </is>
+      </c>
+      <c r="E799" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F799" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G799" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="8" t="inlineStr">
+        <is>
+          <t>prereg.guide_mid.FQ1FY27.bear</t>
+        </is>
+      </c>
+      <c r="B800" s="8" t="n">
+        <v>39600</v>
+      </c>
+      <c r="C800" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D800" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E800" s="8" t="inlineStr">
+        <is>
+          <t>PREREG_A</t>
+        </is>
+      </c>
+      <c r="F800" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G800" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="8" t="inlineStr">
+        <is>
+          <t>derived.guide_weekly.FQ1FY27.bear</t>
+        </is>
+      </c>
+      <c r="B801" s="8" t="n">
+        <v>-0.2135913653920625</v>
+      </c>
+      <c r="C801" s="8" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D801" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E801" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F801" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G801" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="8" t="inlineStr">
+        <is>
+          <t>prereg.guide_mid.FQ1FY27.base</t>
+        </is>
+      </c>
+      <c r="B802" s="8" t="n">
+        <v>48750</v>
+      </c>
+      <c r="C802" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D802" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E802" s="8" t="inlineStr">
+        <is>
+          <t>PREREG_A</t>
+        </is>
+      </c>
+      <c r="F802" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G802" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="8" t="inlineStr">
+        <is>
+          <t>derived.guide_weekly.FQ1FY27.base</t>
+        </is>
+      </c>
+      <c r="B803" s="8" t="n">
+        <v>-0.0318833096682587</v>
+      </c>
+      <c r="C803" s="8" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D803" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E803" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F803" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G803" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="8" t="inlineStr">
+        <is>
+          <t>prereg.guide_mid.FQ1FY27.bull</t>
+        </is>
+      </c>
+      <c r="B804" s="8" t="n">
+        <v>57300</v>
+      </c>
+      <c r="C804" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D804" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E804" s="8" t="inlineStr">
+        <is>
+          <t>PREREG_A</t>
+        </is>
+      </c>
+      <c r="F804" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G804" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="8" t="inlineStr">
+        <is>
+          <t>derived.guide_weekly.FQ1FY27.bull</t>
+        </is>
+      </c>
+      <c r="B805" s="8" t="n">
+        <v>0.1379094637130005</v>
+      </c>
+      <c r="C805" s="8" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D805" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E805" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F805" s="8" t="inlineStr">
+        <is>
+          <t>SRC-FROZEN</t>
+        </is>
+      </c>
+      <c r="G805" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="8" t="inlineStr">
+        <is>
+          <t>guidance.revenue_hi.FQ1FY27</t>
+        </is>
+      </c>
+      <c r="B806" s="8" t="n">
+        <v>63000</v>
+      </c>
+      <c r="C806" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D806" s="8" t="inlineStr">
+        <is>
+          <t>FQ1FY27</t>
+        </is>
+      </c>
+      <c r="E806" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F806" s="8" t="inlineStr">
+        <is>
+          <t>SRC-EX991-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G806" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="8" t="inlineStr">
+        <is>
+          <t>sensitivity.eps.slowdown.FY2027E</t>
+        </is>
+      </c>
+      <c r="B807" s="8" t="n">
+        <v>165.5568709183349</v>
+      </c>
+      <c r="C807" s="8" t="inlineStr">
+        <is>
+          <t>USD_per_share</t>
+        </is>
+      </c>
+      <c r="D807" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E807" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F807" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G807" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="8" t="inlineStr">
+        <is>
+          <t>sensitivity.eps.zero.FY2027E</t>
+        </is>
+      </c>
+      <c r="B808" s="8" t="n">
+        <v>159.6265415679691</v>
+      </c>
+      <c r="C808" s="8" t="inlineStr">
+        <is>
+          <t>USD_per_share</t>
+        </is>
+      </c>
+      <c r="D808" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E808" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F808" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G808" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="8" t="inlineStr">
+        <is>
+          <t>sensitivity.eps.r8.FY2027E</t>
+        </is>
+      </c>
+      <c r="B809" s="8" t="n">
+        <v>170.1393106400569</v>
+      </c>
+      <c r="C809" s="8" t="inlineStr">
+        <is>
+          <t>USD_per_share</t>
+        </is>
+      </c>
+      <c r="D809" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E809" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F809" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G809" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="8" t="inlineStr">
+        <is>
+          <t>sensitivity.eps.original_gm.FY2027E</t>
+        </is>
+      </c>
+      <c r="B810" s="8" t="n">
+        <v>167.4552762620385</v>
+      </c>
+      <c r="C810" s="8" t="inlineStr">
+        <is>
+          <t>USD_per_share</t>
+        </is>
+      </c>
+      <c r="D810" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E810" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F810" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G810" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2024Q1.A</t>
+        </is>
+      </c>
+      <c r="B811" s="8" t="n">
+        <v>1093</v>
+      </c>
+      <c r="C811" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D811" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q1</t>
+        </is>
+      </c>
+      <c r="E811" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F811" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-cba05d3a7684</t>
+        </is>
+      </c>
+      <c r="G811" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2024Q1.A</t>
+        </is>
+      </c>
+      <c r="B812" s="8" t="n">
+        <v>1734</v>
+      </c>
+      <c r="C812" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D812" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q1</t>
+        </is>
+      </c>
+      <c r="E812" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F812" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-cba05d3a7684</t>
+        </is>
+      </c>
+      <c r="G812" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2024Q2.A</t>
+        </is>
+      </c>
+      <c r="B813" s="8" t="n">
+        <v>888</v>
+      </c>
+      <c r="C813" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D813" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q2</t>
+        </is>
+      </c>
+      <c r="E813" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F813" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-a635cd2a7c38</t>
+        </is>
+      </c>
+      <c r="G813" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2024Q2.A</t>
+        </is>
+      </c>
+      <c r="B814" s="8" t="n">
+        <v>1248</v>
+      </c>
+      <c r="C814" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D814" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q2</t>
+        </is>
+      </c>
+      <c r="E814" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F814" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-a635cd2a7c38</t>
+        </is>
+      </c>
+      <c r="G814" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2024Q3.A</t>
+        </is>
+      </c>
+      <c r="B815" s="8" t="n">
+        <v>1113</v>
+      </c>
+      <c r="C815" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D815" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q3</t>
+        </is>
+      </c>
+      <c r="E815" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F815" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-51fa896d882d</t>
+        </is>
+      </c>
+      <c r="G815" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2024Q3.A</t>
+        </is>
+      </c>
+      <c r="B816" s="8" t="n">
+        <v>2057</v>
+      </c>
+      <c r="C816" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D816" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q3</t>
+        </is>
+      </c>
+      <c r="E816" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F816" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-51fa896d882d</t>
+        </is>
+      </c>
+      <c r="G816" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2024Q4.A</t>
+        </is>
+      </c>
+      <c r="B817" s="8" t="n">
+        <v>1215</v>
+      </c>
+      <c r="C817" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D817" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q4</t>
+        </is>
+      </c>
+      <c r="E817" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F817" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-3faad63e6c8e</t>
+        </is>
+      </c>
+      <c r="G817" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2024Q4.A</t>
+        </is>
+      </c>
+      <c r="B818" s="8" t="n">
+        <v>3082</v>
+      </c>
+      <c r="C818" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D818" s="8" t="inlineStr">
+        <is>
+          <t>FY2024Q4</t>
+        </is>
+      </c>
+      <c r="E818" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F818" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-3faad63e6c8e</t>
+        </is>
+      </c>
+      <c r="G818" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2025Q1.A</t>
+        </is>
+      </c>
+      <c r="B819" s="8" t="n">
+        <v>1174</v>
+      </c>
+      <c r="C819" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D819" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q1</t>
+        </is>
+      </c>
+      <c r="E819" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F819" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-f1ece4749d1a</t>
+        </is>
+      </c>
+      <c r="G819" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2025Q1.A</t>
+        </is>
+      </c>
+      <c r="B820" s="8" t="n">
+        <v>3132</v>
+      </c>
+      <c r="C820" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D820" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q1</t>
+        </is>
+      </c>
+      <c r="E820" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F820" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-f1ece4749d1a</t>
+        </is>
+      </c>
+      <c r="G820" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2025Q2.A</t>
+        </is>
+      </c>
+      <c r="B821" s="8" t="n">
+        <v>1190</v>
+      </c>
+      <c r="C821" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D821" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q2</t>
+        </is>
+      </c>
+      <c r="E821" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F821" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-503fbf81dc7f</t>
+        </is>
+      </c>
+      <c r="G821" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2025Q2.A</t>
+        </is>
+      </c>
+      <c r="B822" s="8" t="n">
+        <v>3085</v>
+      </c>
+      <c r="C822" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D822" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q2</t>
+        </is>
+      </c>
+      <c r="E822" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F822" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-503fbf81dc7f</t>
+        </is>
+      </c>
+      <c r="G822" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2025Q3.A</t>
+        </is>
+      </c>
+      <c r="B823" s="8" t="n">
+        <v>1339</v>
+      </c>
+      <c r="C823" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D823" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q3</t>
+        </is>
+      </c>
+      <c r="E823" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F823" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-170cac3d1ae6</t>
+        </is>
+      </c>
+      <c r="G823" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2025Q3.A</t>
+        </is>
+      </c>
+      <c r="B824" s="8" t="n">
+        <v>2660</v>
+      </c>
+      <c r="C824" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D824" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q3</t>
+        </is>
+      </c>
+      <c r="E824" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F824" s="8" t="inlineStr">
+        <is>
+          <t>SRC-GUIDANCE-170cac3d1ae6</t>
+        </is>
+      </c>
+      <c r="G824" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2025Q4.A</t>
+        </is>
+      </c>
+      <c r="B825" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C825" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D825" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q4</t>
+        </is>
+      </c>
+      <c r="E825" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F825" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-34478c62e48f</t>
+        </is>
+      </c>
+      <c r="G825" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2025Q4.A</t>
+        </is>
+      </c>
+      <c r="B826" s="8" t="n">
+        <v>4927</v>
+      </c>
+      <c r="C826" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D826" s="8" t="inlineStr">
+        <is>
+          <t>FY2025Q4</t>
+        </is>
+      </c>
+      <c r="E826" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F826" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-34478c62e48f</t>
+        </is>
+      </c>
+      <c r="G826" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2026Q1.A</t>
+        </is>
+      </c>
+      <c r="B827" s="8" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C827" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D827" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q1</t>
+        </is>
+      </c>
+      <c r="E827" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F827" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-ee2e84a14aef</t>
+        </is>
+      </c>
+      <c r="G827" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2026Q1.A</t>
+        </is>
+      </c>
+      <c r="B828" s="8" t="n">
+        <v>4505</v>
+      </c>
+      <c r="C828" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D828" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q1</t>
+        </is>
+      </c>
+      <c r="E828" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F828" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-ee2e84a14aef</t>
+        </is>
+      </c>
+      <c r="G828" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="8" t="inlineStr">
+        <is>
+          <t>is.opex.FY2026Q2.A</t>
+        </is>
+      </c>
+      <c r="B829" s="8" t="n">
+        <v>1620</v>
+      </c>
+      <c r="C829" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D829" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q2</t>
+        </is>
+      </c>
+      <c r="E829" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F829" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-18c8475fe645</t>
+        </is>
+      </c>
+      <c r="G829" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2026Q2.A</t>
+        </is>
+      </c>
+      <c r="B830" s="8" t="n">
+        <v>5004</v>
+      </c>
+      <c r="C830" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D830" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q2</t>
+        </is>
+      </c>
+      <c r="E830" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F830" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-18c8475fe645</t>
+        </is>
+      </c>
+      <c r="G830" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2026Q3.A</t>
+        </is>
+      </c>
+      <c r="B831" s="8" t="n">
+        <v>7084</v>
+      </c>
+      <c r="C831" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D831" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q3</t>
+        </is>
+      </c>
+      <c r="E831" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F831" s="8" t="inlineStr">
+        <is>
+          <t>SRC-BU-9f7e667a8224</t>
+        </is>
+      </c>
+      <c r="G831" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="8" t="inlineStr">
+        <is>
+          <t>cf.net_capex.FY2026Q4.A</t>
+        </is>
+      </c>
+      <c r="B832" s="8" t="n">
+        <v>10774</v>
+      </c>
+      <c r="C832" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D832" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E832" s="8" t="inlineStr">
+        <is>
+          <t>A-8K</t>
+        </is>
+      </c>
+      <c r="F832" s="8" t="inlineStr">
+        <is>
+          <t>SRC-EX991-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G832" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="8" t="inlineStr">
+        <is>
+          <t>rle.opex.FY2027Q1.base</t>
+        </is>
+      </c>
+      <c r="B833" s="8" t="n">
+        <v>2310</v>
+      </c>
+      <c r="C833" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D833" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q1</t>
+        </is>
+      </c>
+      <c r="E833" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F833" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G833" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="8" t="inlineStr">
+        <is>
+          <t>rle.opex.FY2027Q2.base</t>
+        </is>
+      </c>
+      <c r="B834" s="8" t="n">
+        <v>2413</v>
+      </c>
+      <c r="C834" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D834" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q2</t>
+        </is>
+      </c>
+      <c r="E834" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F834" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G834" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="8" t="inlineStr">
+        <is>
+          <t>rle.opex.FY2027Q3.base</t>
+        </is>
+      </c>
+      <c r="B835" s="8" t="n">
+        <v>2654</v>
+      </c>
+      <c r="C835" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D835" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q3</t>
+        </is>
+      </c>
+      <c r="E835" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F835" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G835" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="8" t="inlineStr">
+        <is>
+          <t>rle.opex.FY2027Q4.base</t>
+        </is>
+      </c>
+      <c r="B836" s="8" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C836" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D836" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q4</t>
+        </is>
+      </c>
+      <c r="E836" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F836" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G836" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="8" t="inlineStr">
+        <is>
+          <t>rle.net_capex.FY2027Q1.base</t>
+        </is>
+      </c>
+      <c r="B837" s="8" t="n">
+        <v>11500</v>
+      </c>
+      <c r="C837" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D837" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q1</t>
+        </is>
+      </c>
+      <c r="E837" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F837" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G837" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="8" t="inlineStr">
+        <is>
+          <t>rle.net_capex.FY2027Q2.base</t>
+        </is>
+      </c>
+      <c r="B838" s="8" t="n">
+        <v>13500</v>
+      </c>
+      <c r="C838" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D838" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q2</t>
+        </is>
+      </c>
+      <c r="E838" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F838" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G838" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="8" t="inlineStr">
+        <is>
+          <t>rle.net_capex.FY2027Q3.base</t>
+        </is>
+      </c>
+      <c r="B839" s="8" t="n">
+        <v>12500</v>
+      </c>
+      <c r="C839" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D839" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q3</t>
+        </is>
+      </c>
+      <c r="E839" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F839" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G839" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="8" t="inlineStr">
+        <is>
+          <t>rle.net_capex.FY2027Q4.base</t>
+        </is>
+      </c>
+      <c r="B840" s="8" t="n">
+        <v>12500</v>
+      </c>
+      <c r="C840" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D840" s="8" t="inlineStr">
+        <is>
+          <t>FY2027Q4</t>
+        </is>
+      </c>
+      <c r="E840" s="8" t="inlineStr">
+        <is>
+          <t>RLE</t>
+        </is>
+      </c>
+      <c r="F840" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G840" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="8" t="inlineStr">
+        <is>
+          <t>bridge.op_amount.revenue.FY2026A_to_FY2027E</t>
+        </is>
+      </c>
+      <c r="B841" s="8" t="n">
+        <v>114290.7123010019</v>
+      </c>
+      <c r="C841" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D841" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E841" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F841" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G841" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="8" t="inlineStr">
+        <is>
+          <t>bridge.op_amount.gm.FY2026A_to_FY2027E</t>
+        </is>
+      </c>
+      <c r="B842" s="8" t="n">
+        <v>14382.25567230563</v>
+      </c>
+      <c r="C842" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D842" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E842" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F842" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G842" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="8" t="inlineStr">
+        <is>
+          <t>bridge.op_amount.opex.FY2026A_to_FY2027E</t>
+        </is>
+      </c>
+      <c r="B843" s="8" t="n">
+        <v>-2189</v>
+      </c>
+      <c r="C843" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D843" s="8" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E843" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F843" s="8" t="inlineStr">
+        <is>
+          <t>SRC-RLE-FY27</t>
+        </is>
+      </c>
+      <c r="G843" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="8" t="inlineStr">
+        <is>
+          <t>sca.contracts.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B844" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="C844" s="8" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D844" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E844" s="8" t="inlineStr">
+        <is>
+          <t>CITED</t>
+        </is>
+      </c>
+      <c r="F844" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G844" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="8" t="inlineStr">
+        <is>
+          <t>sca.revenue_floor.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B845" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="C845" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D845" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E845" s="8" t="inlineStr">
+        <is>
+          <t>CITED</t>
+        </is>
+      </c>
+      <c r="F845" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G845" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="8" t="inlineStr">
+        <is>
+          <t>sca.commitments.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B846" s="8" t="n">
+        <v>32000</v>
+      </c>
+      <c r="C846" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D846" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E846" s="8" t="inlineStr">
+        <is>
+          <t>CITED</t>
+        </is>
+      </c>
+      <c r="F846" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G846" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="8" t="inlineStr">
+        <is>
+          <t>sca.deposits.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B847" s="8" t="n">
+        <v>12700</v>
+      </c>
+      <c r="C847" s="8" t="inlineStr">
+        <is>
+          <t>USD_million</t>
+        </is>
+      </c>
+      <c r="D847" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E847" s="8" t="inlineStr">
+        <is>
+          <t>CITED</t>
+        </is>
+      </c>
+      <c r="F847" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G847" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="8" t="inlineStr">
+        <is>
+          <t>sca.defined_pricing.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B848" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="C848" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D848" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E848" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F848" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G848" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="8" t="inlineStr">
+        <is>
+          <t>sca.market_pricing.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B849" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="C849" s="8" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D849" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E849" s="8" t="inlineStr">
+        <is>
+          <t>CALCULATED</t>
+        </is>
+      </c>
+      <c r="F849" s="8" t="inlineStr">
+        <is>
+          <t>SRC-REMARKS-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G849" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.0.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B850" s="8" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="C850" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D850" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E850" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F850" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G850" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.1.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B851" s="8" t="inlineStr">
+        <is>
+          <t>49,000–51,000</t>
+        </is>
+      </c>
+      <c r="C851" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D851" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E851" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F851" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G851" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.2.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B852" s="8" t="inlineStr">
+        <is>
+          <t>54,229</t>
+        </is>
+      </c>
+      <c r="C852" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D852" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E852" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F852" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G852" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.3.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B853" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C853" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D853" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E853" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F853" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G853" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.4.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B854" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C854" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D854" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E854" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F854" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G854" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.0.5.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B855" s="8" t="inlineStr">
+        <is>
+          <t>적중</t>
+        </is>
+      </c>
+      <c r="C855" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D855" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E855" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F855" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G855" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.0.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B856" s="8" t="inlineStr">
+        <is>
+          <t>GAAP 희석 EPS</t>
+        </is>
+      </c>
+      <c r="C856" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D856" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E856" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F856" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G856" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.1.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B857" s="8" t="inlineStr">
+        <is>
+          <t>29.73–31.73</t>
+        </is>
+      </c>
+      <c r="C857" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D857" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E857" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F857" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G857" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.2.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B858" s="8" t="inlineStr">
+        <is>
+          <t>32.87</t>
+        </is>
+      </c>
+      <c r="C858" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D858" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E858" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F858" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G858" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.3.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B859" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C859" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D859" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E859" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F859" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G859" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.4.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B860" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C860" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D860" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E860" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F860" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G860" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.1.5.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B861" s="8" t="inlineStr">
+        <is>
+          <t>적중</t>
+        </is>
+      </c>
+      <c r="C861" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D861" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E861" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F861" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G861" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.0.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B862" s="8" t="inlineStr">
+        <is>
+          <t>비GAAP 희석 EPS</t>
+        </is>
+      </c>
+      <c r="C862" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D862" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E862" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F862" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G862" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.1.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B863" s="8" t="inlineStr">
+        <is>
+          <t>30.00–32.00</t>
+        </is>
+      </c>
+      <c r="C863" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D863" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E863" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F863" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G863" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.2.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B864" s="8" t="inlineStr">
+        <is>
+          <t>33.42</t>
+        </is>
+      </c>
+      <c r="C864" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D864" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E864" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F864" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G864" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.3.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B865" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C865" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D865" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E865" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F865" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G865" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.4.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B866" s="8" t="inlineStr">
+        <is>
+          <t>ABOVE_HIGH</t>
+        </is>
+      </c>
+      <c r="C866" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D866" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E866" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F866" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G866" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.2.5.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B867" s="8" t="inlineStr">
+        <is>
+          <t>적중</t>
+        </is>
+      </c>
+      <c r="C867" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D867" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E867" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F867" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G867" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.0.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B868" s="8" t="inlineStr">
+        <is>
+          <t>GAAP GM</t>
+        </is>
+      </c>
+      <c r="C868" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D868" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E868" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F868" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G868" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.1.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B869" s="8" t="inlineStr">
+        <is>
+          <t>85.0–87.0%</t>
+        </is>
+      </c>
+      <c r="C869" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D869" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E869" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F869" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G869" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.2.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B870" s="8" t="inlineStr">
+        <is>
+          <t>86.76%</t>
+        </is>
+      </c>
+      <c r="C870" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D870" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E870" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F870" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G870" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.3.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B871" s="8" t="inlineStr">
+        <is>
+          <t>IN_RANGE</t>
+        </is>
+      </c>
+      <c r="C871" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D871" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E871" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F871" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G871" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.4.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B872" s="8" t="inlineStr">
+        <is>
+          <t>IN_RANGE</t>
+        </is>
+      </c>
+      <c r="C872" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D872" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E872" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F872" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G872" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.3.5.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B873" s="8" t="inlineStr">
+        <is>
+          <t>적중</t>
+        </is>
+      </c>
+      <c r="C873" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D873" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E873" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F873" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G873" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.0.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B874" s="8" t="inlineStr">
+        <is>
+          <t>GAAP opex</t>
+        </is>
+      </c>
+      <c r="C874" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D874" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E874" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F874" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G874" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.1.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B875" s="8" t="inlineStr">
+        <is>
+          <t>(선언 없음)</t>
+        </is>
+      </c>
+      <c r="C875" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D875" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E875" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F875" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G875" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.2.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B876" s="8" t="inlineStr">
+        <is>
+          <t>3,296</t>
+        </is>
+      </c>
+      <c r="C876" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D876" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E876" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F876" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G876" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.3.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B877" s="8" t="inlineStr">
+        <is>
+          <t>라벨 없음</t>
+        </is>
+      </c>
+      <c r="C877" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D877" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E877" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F877" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G877" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.4.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B878" s="8" t="inlineStr">
+        <is>
+          <t>(d-1) "IN_RANGE 구성상 동일"</t>
+        </is>
+      </c>
+      <c r="C878" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D878" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E878" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F878" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G878" s="8" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="8" t="inlineStr">
+        <is>
+          <t>scored.verdict.4.5.FQ4FY26</t>
+        </is>
+      </c>
+      <c r="B879" s="8" t="inlineStr">
+        <is>
+          <t>서술 실패</t>
+        </is>
+      </c>
+      <c r="C879" s="8" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D879" s="8" t="inlineStr">
+        <is>
+          <t>FY2026Q4</t>
+        </is>
+      </c>
+      <c r="E879" s="8" t="inlineStr">
+        <is>
+          <t>SCORED</t>
+        </is>
+      </c>
+      <c r="F879" s="8" t="inlineStr">
+        <is>
+          <t>SRC-SCORED-FQ4FY26</t>
+        </is>
+      </c>
+      <c r="G879" s="8" t="inlineStr">
         <is>
           <t>AVAILABLE</t>
         </is>

</xml_diff>